<commit_message>
Correct Southampton localised rankings; add info vs commercial proof layer
Live Southampton-localised SERP checks show firm queries ranking 1-4
(party wall and expert witness pages at #1); product and cost queries
absent even locally. Workbook gains Info vs Commercial and Live SERP
Checks tabs; briefing section 6 rebuilt around the intent split.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013GQ7dsNTJJzb3KGQvEdbJx
</commit_message>
<xml_diff>
--- a/HarrisonClarke_Keyword_Universe.xlsx
+++ b/HarrisonClarke_Keyword_Universe.xlsx
@@ -13,7 +13,9 @@
     <sheet name="Clusters" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Page Plan" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="London Plan" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Recommendations" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Info vs Commercial" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Live SERP Checks" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Recommendations" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'GSC Insights'!$A$1:$C$11</definedName>
@@ -21,7 +23,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Clusters'!$A$1:$E$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Page Plan'!$A$1:$G$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'London Plan'!$A$1:$C$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Recommendations'!$A$1:$D$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Info vs Commercial'!$A$1:$E$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Live SERP Checks'!$A$1:$D$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Recommendations'!$A$1:$D$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -478,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -591,81 +595,95 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>6. Recommendations - the programme in priority order, including measurement/CRM attribution</t>
+          <t>6. Info vs Commercial - per service line: where they rank for information vs where they rank for the commercial terms, with the ideal commercial targets. The proof layer: they rank as a firm and for information, not for the product or the price</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>7. Live SERP Checks - SerpApi results from a Southampton-localised search, 3 Sep 2026. These correct the GSC blended averages: firm queries rank 1-4 locally; product and cost queries are absent even locally</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>8. Recommendations - the programme in priority order, including measurement/CRM attribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>RULES APPLIED</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>- One page per intent: every keyword is owned by exactly one page; no two pages chase the same term</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>- Generic terms go to service/hub pages; specific terms to specific pages; blog supports and links down</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>- Same-vs-separate page decisions follow what page type actually wins the SERP, not word overlap</t>
+          <t>- One page per intent: every keyword is owned by exactly one page; no two pages chase the same term</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>- Generic terms go to service/hub pages; specific terms to specific pages; blog supports and links down</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>- Same-vs-separate page decisions follow what page type actually wins the SERP, not word overlap</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t>- No URL/slug changes to existing ranking pages - titles, H1s, content and internal links only</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>CAVEATS</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>- Volumes are Ahrefs 12-month GB averages; niche terms under ~50/mo carry wide error bars, and seasonality is hidden</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>- CPC shown in USD dollars (Ahrefs reports USD); use as a relative value signal, not a bid estimate</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>- Keyword difficulty (KD) could not be pulled for the full set (Ahrefs API fault on the KD column during research); spot values: 'commercial building survey' KD 2, 'party wall surveyor' KD 14 - both LOW. SERP composition (regional firms, directories) confirms weak-to-moderate competition across the commercial clusters</t>
+          <t>- Volumes are Ahrefs 12-month GB averages; niche terms under ~50/mo carry wide error bars, and seasonality is hidden</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>- CPC shown in USD dollars (Ahrefs reports USD); use as a relative value signal, not a bid estimate</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>- Keyword difficulty (KD) could not be pulled for the full set (Ahrefs API fault on the KD column during research); spot values: 'commercial building survey' KD 2, 'party wall surveyor' KD 14 - both LOW. SERP composition (regional firms, directories) confirms weak-to-moderate competition across the commercial clusters</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>- GSC positions are 6-month averages and lag current state</t>
         </is>
@@ -761,17 +779,17 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Southampton commercial terms sit just off page 1</t>
+          <t>Southampton FIRM queries are already won - locally. Product and cost queries are not, anywhere</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>'building surveyors southampton' pos 11.9 (1,127 impr); 'surveyor southampton' 13.9 (1,598); 'building survey southampton' 15.0 (919); 'chartered surveyor southampton' 18.9 (861). Homepage does the ranking, at pos ~24 avg overall.</t>
+          <t>LIVE localised checks (SerpApi, Southampton location, 3 Sep 2026): 'party wall surveyor southampton' #1; 'expert witness surveyor southampton' #1; 'building surveyor southampton' #2; 'chartered surveyors southampton' #3; 'building survey southampton' #3; 'commercial building survey southampton' #4 (homepage); 'dilapidations surveyor southampton' #6. GSC average positions (11-19) are UK-blended - searchers outside the localisation radius see them lower. BUT even from Southampton: 'house survey southampton', 'house survey cost', 'level 3 survey', 'damp survey southampton' - absent from top 10.</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Near-miss cluster: title/H1 retarget + internal links + homepage merchandising should move 11-19 to 5-8. Local pack is already #1.</t>
+          <t>Corrected thesis: they rank as a FIRM (localised) and for information; they do not rank for the PRODUCT or the PRICE - even at home. The gap is product pages (L2/L3, damp) and cost pages, plus everywhere localisation doesn't rescue them (rest of Hampshire, London, national).</t>
         </is>
       </c>
     </row>
@@ -12590,7 +12608,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>P1. Near-miss positions 11-19 across the board; retargets + rebuilt location pages + Winchester (new).</t>
+          <t>P1, reframed after live checks: Southampton FIRM queries already rank 1-4 on localised SERPs; the local work is product terms ('house survey southampton' absent even locally), the rest of Hampshire (Portsmouth/Winchester pages, where localisation doesn't rescue them), and defending what's won.</t>
         </is>
       </c>
     </row>
@@ -13214,7 +13232,7 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>Title/H1 currently brand-led; add Southampton + chartered surveyor targeting, merchandise (5.0 Google, RICS, two offices), service links with exact anchors</t>
+          <t>Already ranks 2-4 on LOCALISED Southampton SERPs (verified live 3 Sep). Work here is consolidation for non-local searchers (the UK-blended avg is 24): merchandise title/meta (5.0 Google, RICS, two offices) for CTR, and strengthen exact-anchor service links</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -13895,6 +13913,578 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Service line</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Informational: their position today</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Commercial: their position today</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Ideal commercial keywords (the targets)</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Top informational keywords they already own (the ammunition)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Party wall</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>OWNED. 125 non-brand queries, 251 clicks, avg pos 15 (many at 1-8): notice period, award meaning, neighbour scenarios, timescales, consent/dissent, access licence. Best library in the vertical.</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL. 25 queries, 43 clicks, avg pos 16. Localised Southampton: /party-wall/ ranks #1 (verified live). National 'party wall surveyor' pos 26.6 (1,764 impr); 'party wall surveyor cost' pos 28 (1,016 impr, 0 clicks). 'online party wall quote' pos 4.8 - tool nearly winning.</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>party wall surveyor (+cost, +near me, +hampshire, +london &amp; boroughs), rics party wall surveyors, party wall agreement surveyor</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>party wall notice period · what is a party wall award · neighbour started work without agreement · planning an extension under the Act · agreed surveyor guides</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Residential surveys (L2/L3)</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>OWNED. 131 queries, 171 clicks, avg pos 25 (decision content at 7-9): level 2 vs level 3 (3,283 + 3,070 impr), what each covers, surveyor missed a defect.</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>ABSENT. 51 commercial queries, 27,682 impressions, FOUR clicks, avg pos 43. Every cost query unranked (house survey cost pos 34.5 on 3,178 impr). Even localised: 'house survey southampton' and 'level 3 survey' - not in top 10 from Southampton.</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>level 2 survey, level 3 survey, homebuyers survey (all variants), house survey cost, level 2/3 survey cost, house survey southampton, building survey winchester/portsmouth</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>level 2 vs level 3 survey (their best asset) · what does a level 2/3 cover · when your surveyor misses a defect · red flags on a house survey</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Defect &amp; damp</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>OWNED. 149 queries, 256 clicks, avg pos 19 (cracks pos 2.8, damp meter pos 2.2-5.6, wall tie failure, timber frame, RAAC).</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>ABSENT. ~0 commercial capture. 'damp survey southampton' top 10: treatment firms and independent damp specialists - no Harrison Clarke. Their content pre-sells a service page that doesn't target the demand.</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>damp survey (+cost, +southampton), independent damp survey, structural survey cost, subsidence survey, single defect report phrasing</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>using a damp meter · cracks in buildings when to worry · thermal movement cracks · wall tie failure · can woodworm damage your home · RAAC identification</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Dilapidations</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL. 54 queries, 28 clicks, avg pos 37: what is a schedule, interim schedule purpose, received-a-schedule guides, London disputes post.</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>ABSENT. 12 queries, 4 clicks, avg pos 36. 'dilapidations surveyor' pos 38 (589 impr); 'dilapidation survey' pos 80; 'schedule of dilapidations' pos 13.9 on 2,558 impr = nearly there; 'dilapidations surveyor london' pos 9.8 via blog. Localised Southampton: #6.</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>dilapidations surveyor (+london, +hampshire, +southampton), dilapidation survey/report, schedule of dilapidations, commercial property dilapidations, office/industrial dilapidations</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>what is the purpose of an interim schedule · received a schedule of dilapidations don't panic · how to resolve dilapidations disputes in London (the pos-9.8 asset)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Commercial surveys / TDD</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>THIN. 5 queries, 2 clicks: the comprehensive guide (ranks pos 8 for the head term), what a survey includes (pos 53).</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>ABSENT. 'commercial building surveyors' pos 18 (895 impr, 0 clicks); 'commercial building surveyor' pos 29. Service page pos 30 on its own term (KD 2). Localised: homepage #4 - the wrong page ranks.</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>commercial building survey (+cost), commercial building surveyor, commercial property survey, technical due diligence, pre acquisition survey (rics)</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>a comprehensive guide to commercial building surveys (repoint at service page) · what does a commercial building survey include</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Expert witness</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>OWNED (niche). CPR-35 explainer pos 9.2 (8,658 impr), declaration &amp; statement of truth pos 10, role-of guides.</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>ABSENT nationally, WON locally. 'expert witness building surveyor' pos 22.6 (597 impr, 0 clicks); page pos 27. But 'expert witness surveyor southampton' - #1 live. The £300k ambition needs the national/London terms.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>expert witness building surveyor, construction expert witness (+services), building expert witness, property expert witness, expert witness surveyor london, fees content</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>what is CPR 35 · the declaration and statement of truth · appointing a building surveyor as expert witness · role of expert witness in construction</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Project services</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>OWNED (adjacent). 49 queries, 56 clicks, avg pos 8.1 - ALL informational: LADs (pos 1, 2,900 vol), CDM meaning, JCT content.</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>NON-EXISTENT. Zero commercial project-services queries captured. CA/EA page pos 16.7 on 958 impr; CDM page pos 20. The demand that exists (cdm advisor, contract administration, employers agent, principal designer services) is modest but uncontested-adjacent.</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>contract administration (construction), employers agent, cdm advisor (+services), principal designer services/building regulations, project monitoring surveyor</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>what are LADs (pos 1 - their biggest informational asset) · CDM regulations explained · JCT content</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Bonus: reinstatement cost</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>ACCIDENTAL. ~6,700 impressions across 'reinstatement cost assessment' variants at pos 24-77 with ~1 click - demand they attract without a service page.</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>NOT TARGETED. If they offer RCAs (most building surveyors do), this is a free service line: real demand, weak coverage, insurance-driven recurring work.</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>reinstatement cost assessment (+rics, +building), reinstatement cost valuation</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>ASK TIM: do they offer reinstatement cost assessments? If yes - new service page, near-instant fit</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Query</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Searched from</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Harrison Clarke result</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Who wins instead / notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>party wall surveyor southampton</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Southampton (localised)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>#1 - /party-wall/</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Also Faye's FPWS listing at #9. WON.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>expert witness surveyor southampton</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Southampton (localised)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>#1 - /expert-witness/</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>WON locally; national EW terms remain the gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>building surveyor southampton</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Southampton (localised)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>#2 - homepage</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>ricsfirms directory #1. WON.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>chartered surveyors southampton</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Southampton (localised)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>#3 - homepage</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Trinity Rose #1, ricsfirms #2 (HC named in its snippet). WON.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>building survey southampton</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Southampton (localised)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>#3 - homepage</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Directories + Trinity Rose above. WON - but homepage, not a survey page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>commercial building survey southampton</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Southampton (localised)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>#4 - homepage</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Bressummer Ark's dedicated page #2; SC Building Consultancy #6. Present, wrong page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>dilapidations surveyor southampton</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Southampton (localised)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>#6 - /schedule-of-dilapidations/ (+ YouTube #8)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>SC Building Consultancy's dedicated Southampton dilaps page #2. Beatable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>house survey southampton</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Southampton (localised)</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>NOT in top 10</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Directories, Countrywide, Nuven, local one-man firms. The PRODUCT term fails even at home.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>house survey cost</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Southampton (localised)</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>NOT in top 10</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>RICS, MoneySuperMarket, Nationwide, HOA, Checkatrade + Novello Surveyors' cost blog (#10 - proof a firm can rank). No HC cost page exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>level 3 survey</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Southampton (localised)</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>NOT in top 10</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>L&amp;G, RICS, e.surv, Peter Barry's L3 service page (#6 - proof a firm's product page can rank). No dedicated HC L3 page exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>damp survey southampton</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Southampton (localised)</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>NOT in top 10</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Checkatrade + treatment firms + independent damp specialists. Independent-surveyor angle unclaimed by HC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>dilapidations surveyor london</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>UK (national)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>#8 - blog post</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>SHW, TD-RE, Bradley Mason, Easton Bevins - all dedicated London dilaps service pages. No HC service page exists.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D13"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -14032,12 +14622,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Southampton near-miss push</t>
+          <t>Southampton: defend the firm terms, win the product terms</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Homepage + residential hub retargets, location page rebuilds (Portsmouth, Hampshire), NEW Winchester page. Positions 11-19 across ~8,000 impr/mo of local commercial queries.</t>
+          <t>Firm queries already rank 1-4 on localised SERPs (verified live). The work: product pages (L2/L3, damp, house survey southampton - absent even locally), rest-of-Hampshire pages where localisation doesn't rescue them (Portsmouth rebuild, NEW Winchester), and CTR merchandising on the terms already won.</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">

</xml_diff>